<commit_message>
Remove AI branding from README
</commit_message>
<xml_diff>
--- a/outputs/etr_risk_report.xlsx
+++ b/outputs/etr_risk_report.xlsx
@@ -619,7 +619,7 @@
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>ai_reviewer_comment</t>
+          <t>reviewer_comment</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>ai_reviewer_comment</t>
+          <t>reviewer_comment</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>ai_reviewer_comment</t>
+          <t>reviewer_comment</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">

</xml_diff>